<commit_message>
update 1000 cus experiment 1-full
</commit_message>
<xml_diff>
--- a/master-slave/outputs/exp1-full/runs.xlsx
+++ b/master-slave/outputs/exp1-full/runs.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K1201"/>
+  <dimension ref="A1:K1255"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -44296,9 +44296,15 @@
       <c r="G1125" t="n">
         <v>1773.817056086561</v>
       </c>
+      <c r="H1125" t="n">
+        <v>1761.180277491662</v>
+      </c>
       <c r="I1125" t="n">
         <v>1754.17297722392</v>
       </c>
+      <c r="J1125" t="n">
+        <v>58304049011</v>
+      </c>
       <c r="K1125" t="n">
         <v>60823425788</v>
       </c>
@@ -44329,9 +44335,15 @@
       <c r="G1126" t="n">
         <v>1773.817056086561</v>
       </c>
+      <c r="H1126" t="n">
+        <v>1778.484926842881</v>
+      </c>
       <c r="I1126" t="n">
         <v>1771.655567491526</v>
       </c>
+      <c r="J1126" t="n">
+        <v>58751249777</v>
+      </c>
       <c r="K1126" t="n">
         <v>60639155482</v>
       </c>
@@ -44339,7 +44351,7 @@
     <row r="1127">
       <c r="A1127" t="inlineStr">
         <is>
-          <t>1000.10.2</t>
+          <t>1000.10.1</t>
         </is>
       </c>
       <c r="B1127" t="n">
@@ -44354,31 +44366,25 @@
         <v>4500</v>
       </c>
       <c r="E1127" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F1127" t="n">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="G1127" t="n">
-        <v>1761.739356115498</v>
+        <v>1773.817056086561</v>
       </c>
       <c r="H1127" t="n">
-        <v>1748.663684856989</v>
-      </c>
-      <c r="I1127" t="n">
-        <v>1742.937265530643</v>
+        <v>1779.502525723669</v>
       </c>
       <c r="J1127" t="n">
-        <v>58812269481</v>
-      </c>
-      <c r="K1127" t="n">
-        <v>61315522970</v>
+        <v>58545801955</v>
       </c>
     </row>
     <row r="1128">
       <c r="A1128" t="inlineStr">
         <is>
-          <t>1000.10.2</t>
+          <t>1000.10.1</t>
         </is>
       </c>
       <c r="B1128" t="n">
@@ -44393,31 +44399,25 @@
         <v>4500</v>
       </c>
       <c r="E1128" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F1128" t="n">
-        <v>200</v>
+        <v>700</v>
       </c>
       <c r="G1128" t="n">
-        <v>1761.739356115498</v>
+        <v>1773.817056086561</v>
       </c>
       <c r="H1128" t="n">
-        <v>1753.0778443804</v>
-      </c>
-      <c r="I1128" t="n">
-        <v>1743.318234245733</v>
+        <v>1780.589189225288</v>
       </c>
       <c r="J1128" t="n">
-        <v>58793302310</v>
-      </c>
-      <c r="K1128" t="n">
-        <v>61145794679</v>
+        <v>58392419534</v>
       </c>
     </row>
     <row r="1129">
       <c r="A1129" t="inlineStr">
         <is>
-          <t>1000.10.2</t>
+          <t>1000.10.1</t>
         </is>
       </c>
       <c r="B1129" t="n">
@@ -44432,31 +44432,25 @@
         <v>4500</v>
       </c>
       <c r="E1129" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F1129" t="n">
-        <v>300</v>
+        <v>800</v>
       </c>
       <c r="G1129" t="n">
-        <v>1761.739356115498</v>
+        <v>1773.817056086561</v>
       </c>
       <c r="H1129" t="n">
-        <v>1733.720824201108</v>
-      </c>
-      <c r="I1129" t="n">
-        <v>1740.796072994495</v>
+        <v>1776.968992761991</v>
       </c>
       <c r="J1129" t="n">
-        <v>58755870420</v>
-      </c>
-      <c r="K1129" t="n">
-        <v>61540538472</v>
+        <v>58840628439</v>
       </c>
     </row>
     <row r="1130">
       <c r="A1130" t="inlineStr">
         <is>
-          <t>1000.10.2</t>
+          <t>1000.10.1</t>
         </is>
       </c>
       <c r="B1130" t="n">
@@ -44471,25 +44465,25 @@
         <v>4500</v>
       </c>
       <c r="E1130" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F1130" t="n">
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="G1130" t="n">
-        <v>1761.739356115498</v>
-      </c>
-      <c r="I1130" t="n">
-        <v>1737.854667478625</v>
-      </c>
-      <c r="K1130" t="n">
-        <v>60993567814</v>
+        <v>1773.817056086561</v>
+      </c>
+      <c r="H1130" t="n">
+        <v>1778.529257677659</v>
+      </c>
+      <c r="J1130" t="n">
+        <v>58670966138</v>
       </c>
     </row>
     <row r="1131">
       <c r="A1131" t="inlineStr">
         <is>
-          <t>1000.10.2</t>
+          <t>1000.10.1</t>
         </is>
       </c>
       <c r="B1131" t="n">
@@ -44504,25 +44498,25 @@
         <v>4500</v>
       </c>
       <c r="E1131" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F1131" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G1131" t="n">
-        <v>1761.739356115498</v>
-      </c>
-      <c r="I1131" t="n">
-        <v>1736.731224875093</v>
-      </c>
-      <c r="K1131" t="n">
-        <v>61288617891</v>
+        <v>1773.817056086561</v>
+      </c>
+      <c r="H1131" t="n">
+        <v>1773.755316878341</v>
+      </c>
+      <c r="J1131" t="n">
+        <v>58201667902</v>
       </c>
     </row>
     <row r="1132">
       <c r="A1132" t="inlineStr">
         <is>
-          <t>1000.10.3</t>
+          <t>1000.10.2</t>
         </is>
       </c>
       <c r="B1132" t="n">
@@ -44543,25 +44537,25 @@
         <v>100</v>
       </c>
       <c r="G1132" t="n">
-        <v>1748.302363736126</v>
+        <v>1761.739356115498</v>
       </c>
       <c r="H1132" t="n">
-        <v>1764.908007473116</v>
+        <v>1748.663684856989</v>
       </c>
       <c r="I1132" t="n">
-        <v>1760.654491641879</v>
+        <v>1742.937265530643</v>
       </c>
       <c r="J1132" t="n">
-        <v>58893253402</v>
+        <v>58812269481</v>
       </c>
       <c r="K1132" t="n">
-        <v>61164450752</v>
+        <v>61315522970</v>
       </c>
     </row>
     <row r="1133">
       <c r="A1133" t="inlineStr">
         <is>
-          <t>1000.10.3</t>
+          <t>1000.10.2</t>
         </is>
       </c>
       <c r="B1133" t="n">
@@ -44582,25 +44576,25 @@
         <v>200</v>
       </c>
       <c r="G1133" t="n">
-        <v>1748.302363736126</v>
+        <v>1761.739356115498</v>
       </c>
       <c r="H1133" t="n">
-        <v>1745.232279618789</v>
+        <v>1753.0778443804</v>
       </c>
       <c r="I1133" t="n">
-        <v>1749.202199750996</v>
+        <v>1743.318234245733</v>
       </c>
       <c r="J1133" t="n">
-        <v>59297447103</v>
+        <v>58793302310</v>
       </c>
       <c r="K1133" t="n">
-        <v>61614359995</v>
+        <v>61145794679</v>
       </c>
     </row>
     <row r="1134">
       <c r="A1134" t="inlineStr">
         <is>
-          <t>1000.10.3</t>
+          <t>1000.10.2</t>
         </is>
       </c>
       <c r="B1134" t="n">
@@ -44621,25 +44615,25 @@
         <v>300</v>
       </c>
       <c r="G1134" t="n">
-        <v>1748.302363736126</v>
+        <v>1761.739356115498</v>
       </c>
       <c r="H1134" t="n">
-        <v>1753.412563400108</v>
+        <v>1733.720824201108</v>
       </c>
       <c r="I1134" t="n">
-        <v>1746.964360199898</v>
+        <v>1740.796072994495</v>
       </c>
       <c r="J1134" t="n">
-        <v>59138365297</v>
+        <v>58755870420</v>
       </c>
       <c r="K1134" t="n">
-        <v>61283413634</v>
+        <v>61540538472</v>
       </c>
     </row>
     <row r="1135">
       <c r="A1135" t="inlineStr">
         <is>
-          <t>1000.10.3</t>
+          <t>1000.10.2</t>
         </is>
       </c>
       <c r="B1135" t="n">
@@ -44660,19 +44654,25 @@
         <v>400</v>
       </c>
       <c r="G1135" t="n">
-        <v>1748.302363736126</v>
+        <v>1761.739356115498</v>
+      </c>
+      <c r="H1135" t="n">
+        <v>1737.922114024622</v>
       </c>
       <c r="I1135" t="n">
-        <v>1727.103620106004</v>
+        <v>1737.854667478625</v>
+      </c>
+      <c r="J1135" t="n">
+        <v>58672060974</v>
       </c>
       <c r="K1135" t="n">
-        <v>61203432562</v>
+        <v>60993567814</v>
       </c>
     </row>
     <row r="1136">
       <c r="A1136" t="inlineStr">
         <is>
-          <t>1000.10.3</t>
+          <t>1000.10.2</t>
         </is>
       </c>
       <c r="B1136" t="n">
@@ -44693,19 +44693,25 @@
         <v>500</v>
       </c>
       <c r="G1136" t="n">
-        <v>1748.302363736126</v>
+        <v>1761.739356115498</v>
+      </c>
+      <c r="H1136" t="n">
+        <v>1740.933155221184</v>
       </c>
       <c r="I1136" t="n">
-        <v>1757.041532870469</v>
+        <v>1736.731224875093</v>
+      </c>
+      <c r="J1136" t="n">
+        <v>58838309757</v>
       </c>
       <c r="K1136" t="n">
-        <v>61084811192</v>
+        <v>61288617891</v>
       </c>
     </row>
     <row r="1137">
       <c r="A1137" t="inlineStr">
         <is>
-          <t>1000.10.4</t>
+          <t>1000.10.2</t>
         </is>
       </c>
       <c r="B1137" t="n">
@@ -44720,31 +44726,25 @@
         <v>4500</v>
       </c>
       <c r="E1137" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F1137" t="n">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="G1137" t="n">
-        <v>1745.548800328407</v>
+        <v>1761.739356115498</v>
       </c>
       <c r="H1137" t="n">
-        <v>1724.519140458432</v>
-      </c>
-      <c r="I1137" t="n">
-        <v>1730.539238991366</v>
+        <v>1749.902760580146</v>
       </c>
       <c r="J1137" t="n">
-        <v>59718078278</v>
-      </c>
-      <c r="K1137" t="n">
-        <v>62112379253</v>
+        <v>59048644443</v>
       </c>
     </row>
     <row r="1138">
       <c r="A1138" t="inlineStr">
         <is>
-          <t>1000.10.4</t>
+          <t>1000.10.2</t>
         </is>
       </c>
       <c r="B1138" t="n">
@@ -44759,31 +44759,25 @@
         <v>4500</v>
       </c>
       <c r="E1138" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F1138" t="n">
-        <v>200</v>
+        <v>700</v>
       </c>
       <c r="G1138" t="n">
-        <v>1745.548800328407</v>
+        <v>1761.739356115498</v>
       </c>
       <c r="H1138" t="n">
-        <v>1727.349755495702</v>
-      </c>
-      <c r="I1138" t="n">
-        <v>1728.751156453611</v>
+        <v>1749.994326897618</v>
       </c>
       <c r="J1138" t="n">
-        <v>59700888210</v>
-      </c>
-      <c r="K1138" t="n">
-        <v>61935437391</v>
+        <v>58807458647</v>
       </c>
     </row>
     <row r="1139">
       <c r="A1139" t="inlineStr">
         <is>
-          <t>1000.10.4</t>
+          <t>1000.10.2</t>
         </is>
       </c>
       <c r="B1139" t="n">
@@ -44798,31 +44792,25 @@
         <v>4500</v>
       </c>
       <c r="E1139" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F1139" t="n">
-        <v>300</v>
+        <v>800</v>
       </c>
       <c r="G1139" t="n">
-        <v>1745.548800328407</v>
+        <v>1761.739356115498</v>
       </c>
       <c r="H1139" t="n">
-        <v>1716.732256778813</v>
-      </c>
-      <c r="I1139" t="n">
-        <v>1720.205219492753</v>
+        <v>1754.023937686556</v>
       </c>
       <c r="J1139" t="n">
-        <v>59511032983</v>
-      </c>
-      <c r="K1139" t="n">
-        <v>62016875497</v>
+        <v>58601057445</v>
       </c>
     </row>
     <row r="1140">
       <c r="A1140" t="inlineStr">
         <is>
-          <t>1000.10.4</t>
+          <t>1000.10.2</t>
         </is>
       </c>
       <c r="B1140" t="n">
@@ -44837,25 +44825,25 @@
         <v>4500</v>
       </c>
       <c r="E1140" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F1140" t="n">
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="G1140" t="n">
-        <v>1745.548800328407</v>
-      </c>
-      <c r="I1140" t="n">
-        <v>1729.212291366578</v>
-      </c>
-      <c r="K1140" t="n">
-        <v>62343039325</v>
+        <v>1761.739356115498</v>
+      </c>
+      <c r="H1140" t="n">
+        <v>1750.916803846784</v>
+      </c>
+      <c r="J1140" t="n">
+        <v>58802514505</v>
       </c>
     </row>
     <row r="1141">
       <c r="A1141" t="inlineStr">
         <is>
-          <t>1000.10.4</t>
+          <t>1000.10.2</t>
         </is>
       </c>
       <c r="B1141" t="n">
@@ -44870,25 +44858,25 @@
         <v>4500</v>
       </c>
       <c r="E1141" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F1141" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G1141" t="n">
-        <v>1745.548800328407</v>
-      </c>
-      <c r="I1141" t="n">
-        <v>1725.545009636343</v>
-      </c>
-      <c r="K1141" t="n">
-        <v>62305690457</v>
+        <v>1761.739356115498</v>
+      </c>
+      <c r="H1141" t="n">
+        <v>1758.879779620557</v>
+      </c>
+      <c r="J1141" t="n">
+        <v>58863099099</v>
       </c>
     </row>
     <row r="1142">
       <c r="A1142" t="inlineStr">
         <is>
-          <t>1000.20.1</t>
+          <t>1000.10.3</t>
         </is>
       </c>
       <c r="B1142" t="n">
@@ -44909,25 +44897,25 @@
         <v>100</v>
       </c>
       <c r="G1142" t="n">
-        <v>3708.541021396037</v>
+        <v>1748.302363736126</v>
       </c>
       <c r="H1142" t="n">
-        <v>3711.484141374198</v>
+        <v>1764.908007473116</v>
       </c>
       <c r="I1142" t="n">
-        <v>3709.684088929843</v>
+        <v>1760.654491641879</v>
       </c>
       <c r="J1142" t="n">
-        <v>54539220721</v>
+        <v>58893253402</v>
       </c>
       <c r="K1142" t="n">
-        <v>57058097271</v>
+        <v>61164450752</v>
       </c>
     </row>
     <row r="1143">
       <c r="A1143" t="inlineStr">
         <is>
-          <t>1000.20.1</t>
+          <t>1000.10.3</t>
         </is>
       </c>
       <c r="B1143" t="n">
@@ -44948,25 +44936,25 @@
         <v>200</v>
       </c>
       <c r="G1143" t="n">
-        <v>3708.541021396037</v>
+        <v>1748.302363736126</v>
       </c>
       <c r="H1143" t="n">
-        <v>3717.075646092836</v>
+        <v>1745.232279618789</v>
       </c>
       <c r="I1143" t="n">
-        <v>3712.684249728848</v>
+        <v>1749.202199750996</v>
       </c>
       <c r="J1143" t="n">
-        <v>54746244345</v>
+        <v>59297447103</v>
       </c>
       <c r="K1143" t="n">
-        <v>57502335211</v>
+        <v>61614359995</v>
       </c>
     </row>
     <row r="1144">
       <c r="A1144" t="inlineStr">
         <is>
-          <t>1000.20.1</t>
+          <t>1000.10.3</t>
         </is>
       </c>
       <c r="B1144" t="n">
@@ -44987,25 +44975,25 @@
         <v>300</v>
       </c>
       <c r="G1144" t="n">
-        <v>3708.541021396037</v>
+        <v>1748.302363736126</v>
       </c>
       <c r="H1144" t="n">
-        <v>3709.542619220546</v>
+        <v>1753.412563400108</v>
       </c>
       <c r="I1144" t="n">
-        <v>3710.003790441718</v>
+        <v>1746.964360199898</v>
       </c>
       <c r="J1144" t="n">
-        <v>54542720537</v>
+        <v>59138365297</v>
       </c>
       <c r="K1144" t="n">
-        <v>57084344927</v>
+        <v>61283413634</v>
       </c>
     </row>
     <row r="1145">
       <c r="A1145" t="inlineStr">
         <is>
-          <t>1000.20.1</t>
+          <t>1000.10.3</t>
         </is>
       </c>
       <c r="B1145" t="n">
@@ -45026,19 +45014,25 @@
         <v>400</v>
       </c>
       <c r="G1145" t="n">
-        <v>3708.541021396037</v>
+        <v>1748.302363736126</v>
+      </c>
+      <c r="H1145" t="n">
+        <v>1737.817941207517</v>
       </c>
       <c r="I1145" t="n">
-        <v>3715.817786494159</v>
+        <v>1727.103620106004</v>
+      </c>
+      <c r="J1145" t="n">
+        <v>58927389309</v>
       </c>
       <c r="K1145" t="n">
-        <v>57407086972</v>
+        <v>61203432562</v>
       </c>
     </row>
     <row r="1146">
       <c r="A1146" t="inlineStr">
         <is>
-          <t>1000.20.1</t>
+          <t>1000.10.3</t>
         </is>
       </c>
       <c r="B1146" t="n">
@@ -45059,19 +45053,25 @@
         <v>500</v>
       </c>
       <c r="G1146" t="n">
-        <v>3708.541021396037</v>
+        <v>1748.302363736126</v>
+      </c>
+      <c r="H1146" t="n">
+        <v>1764.732542053042</v>
       </c>
       <c r="I1146" t="n">
-        <v>3724.648872747662</v>
+        <v>1757.041532870469</v>
+      </c>
+      <c r="J1146" t="n">
+        <v>59185636772</v>
       </c>
       <c r="K1146" t="n">
-        <v>57367898275</v>
+        <v>61084811192</v>
       </c>
     </row>
     <row r="1147">
       <c r="A1147" t="inlineStr">
         <is>
-          <t>1000.20.2</t>
+          <t>1000.10.3</t>
         </is>
       </c>
       <c r="B1147" t="n">
@@ -45086,31 +45086,25 @@
         <v>4500</v>
       </c>
       <c r="E1147" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F1147" t="n">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="G1147" t="n">
-        <v>3768.103517429845</v>
+        <v>1748.302363736126</v>
       </c>
       <c r="H1147" t="n">
-        <v>3718.334914449701</v>
-      </c>
-      <c r="I1147" t="n">
-        <v>3707.205779416522</v>
+        <v>1754.200214247582</v>
       </c>
       <c r="J1147" t="n">
-        <v>54522257604</v>
-      </c>
-      <c r="K1147" t="n">
-        <v>56748923914</v>
+        <v>59034087754</v>
       </c>
     </row>
     <row r="1148">
       <c r="A1148" t="inlineStr">
         <is>
-          <t>1000.20.2</t>
+          <t>1000.10.3</t>
         </is>
       </c>
       <c r="B1148" t="n">
@@ -45125,31 +45119,25 @@
         <v>4500</v>
       </c>
       <c r="E1148" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F1148" t="n">
-        <v>200</v>
+        <v>700</v>
       </c>
       <c r="G1148" t="n">
-        <v>3768.103517429845</v>
+        <v>1748.302363736126</v>
       </c>
       <c r="H1148" t="n">
-        <v>3712.59434092089</v>
-      </c>
-      <c r="I1148" t="n">
-        <v>3688.571250633831</v>
+        <v>1753.291016025567</v>
       </c>
       <c r="J1148" t="n">
-        <v>54713477727</v>
-      </c>
-      <c r="K1148" t="n">
-        <v>57558889306</v>
+        <v>59078203622</v>
       </c>
     </row>
     <row r="1149">
       <c r="A1149" t="inlineStr">
         <is>
-          <t>1000.20.2</t>
+          <t>1000.10.3</t>
         </is>
       </c>
       <c r="B1149" t="n">
@@ -45164,31 +45152,25 @@
         <v>4500</v>
       </c>
       <c r="E1149" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F1149" t="n">
-        <v>300</v>
+        <v>800</v>
       </c>
       <c r="G1149" t="n">
-        <v>3768.103517429845</v>
+        <v>1748.302363736126</v>
       </c>
       <c r="H1149" t="n">
-        <v>3730.776752188581</v>
-      </c>
-      <c r="I1149" t="n">
-        <v>3725.00272664874</v>
+        <v>1751.161091824358</v>
       </c>
       <c r="J1149" t="n">
-        <v>54778015958</v>
-      </c>
-      <c r="K1149" t="n">
-        <v>57374818287</v>
+        <v>58893426637</v>
       </c>
     </row>
     <row r="1150">
       <c r="A1150" t="inlineStr">
         <is>
-          <t>1000.20.2</t>
+          <t>1000.10.3</t>
         </is>
       </c>
       <c r="B1150" t="n">
@@ -45203,25 +45185,25 @@
         <v>4500</v>
       </c>
       <c r="E1150" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F1150" t="n">
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="G1150" t="n">
-        <v>3768.103517429845</v>
-      </c>
-      <c r="I1150" t="n">
-        <v>3731.317629012444</v>
-      </c>
-      <c r="K1150" t="n">
-        <v>57923996919</v>
+        <v>1748.302363736126</v>
+      </c>
+      <c r="H1150" t="n">
+        <v>1756.17380017651</v>
+      </c>
+      <c r="J1150" t="n">
+        <v>58421769698</v>
       </c>
     </row>
     <row r="1151">
       <c r="A1151" t="inlineStr">
         <is>
-          <t>1000.20.2</t>
+          <t>1000.10.3</t>
         </is>
       </c>
       <c r="B1151" t="n">
@@ -45236,25 +45218,25 @@
         <v>4500</v>
       </c>
       <c r="E1151" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F1151" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G1151" t="n">
-        <v>3768.103517429845</v>
-      </c>
-      <c r="I1151" t="n">
-        <v>3698.256619021398</v>
-      </c>
-      <c r="K1151" t="n">
-        <v>57292622262</v>
+        <v>1748.302363736126</v>
+      </c>
+      <c r="H1151" t="n">
+        <v>1745.771127390251</v>
+      </c>
+      <c r="J1151" t="n">
+        <v>58948301864</v>
       </c>
     </row>
     <row r="1152">
       <c r="A1152" t="inlineStr">
         <is>
-          <t>1000.20.3</t>
+          <t>1000.10.4</t>
         </is>
       </c>
       <c r="B1152" t="n">
@@ -45275,25 +45257,25 @@
         <v>100</v>
       </c>
       <c r="G1152" t="n">
-        <v>3734.724211492563</v>
+        <v>1745.548800328407</v>
       </c>
       <c r="H1152" t="n">
-        <v>3675.718557688236</v>
+        <v>1724.519140458432</v>
       </c>
       <c r="I1152" t="n">
-        <v>3679.378142308556</v>
+        <v>1730.539238991366</v>
       </c>
       <c r="J1152" t="n">
-        <v>55234934660</v>
+        <v>59718078278</v>
       </c>
       <c r="K1152" t="n">
-        <v>57888578439</v>
+        <v>62112379253</v>
       </c>
     </row>
     <row r="1153">
       <c r="A1153" t="inlineStr">
         <is>
-          <t>1000.20.3</t>
+          <t>1000.10.4</t>
         </is>
       </c>
       <c r="B1153" t="n">
@@ -45314,25 +45296,25 @@
         <v>200</v>
       </c>
       <c r="G1153" t="n">
-        <v>3734.724211492563</v>
+        <v>1745.548800328407</v>
       </c>
       <c r="H1153" t="n">
-        <v>3671.040088594132</v>
+        <v>1727.349755495702</v>
       </c>
       <c r="I1153" t="n">
-        <v>3661.716562358774</v>
+        <v>1728.751156453611</v>
       </c>
       <c r="J1153" t="n">
-        <v>55008199465</v>
+        <v>59700888210</v>
       </c>
       <c r="K1153" t="n">
-        <v>58027715698</v>
+        <v>61935437391</v>
       </c>
     </row>
     <row r="1154">
       <c r="A1154" t="inlineStr">
         <is>
-          <t>1000.20.3</t>
+          <t>1000.10.4</t>
         </is>
       </c>
       <c r="B1154" t="n">
@@ -45353,25 +45335,25 @@
         <v>300</v>
       </c>
       <c r="G1154" t="n">
-        <v>3734.724211492563</v>
+        <v>1745.548800328407</v>
       </c>
       <c r="H1154" t="n">
-        <v>3679.658407988477</v>
+        <v>1716.732256778813</v>
       </c>
       <c r="I1154" t="n">
-        <v>3666.047778478794</v>
+        <v>1720.205219492753</v>
       </c>
       <c r="J1154" t="n">
-        <v>54859740947</v>
+        <v>59511032983</v>
       </c>
       <c r="K1154" t="n">
-        <v>57560856429</v>
+        <v>62016875497</v>
       </c>
     </row>
     <row r="1155">
       <c r="A1155" t="inlineStr">
         <is>
-          <t>1000.20.3</t>
+          <t>1000.10.4</t>
         </is>
       </c>
       <c r="B1155" t="n">
@@ -45392,19 +45374,25 @@
         <v>400</v>
       </c>
       <c r="G1155" t="n">
-        <v>3734.724211492563</v>
+        <v>1745.548800328407</v>
+      </c>
+      <c r="H1155" t="n">
+        <v>1736.421105443752</v>
       </c>
       <c r="I1155" t="n">
-        <v>3671.922246025872</v>
+        <v>1729.212291366578</v>
+      </c>
+      <c r="J1155" t="n">
+        <v>59616870738</v>
       </c>
       <c r="K1155" t="n">
-        <v>57868215020</v>
+        <v>62343039325</v>
       </c>
     </row>
     <row r="1156">
       <c r="A1156" t="inlineStr">
         <is>
-          <t>1000.20.3</t>
+          <t>1000.10.4</t>
         </is>
       </c>
       <c r="B1156" t="n">
@@ -45425,19 +45413,25 @@
         <v>500</v>
       </c>
       <c r="G1156" t="n">
-        <v>3734.724211492563</v>
+        <v>1745.548800328407</v>
+      </c>
+      <c r="H1156" t="n">
+        <v>1738.975850367712</v>
       </c>
       <c r="I1156" t="n">
-        <v>3692.032536338156</v>
+        <v>1725.545009636343</v>
+      </c>
+      <c r="J1156" t="n">
+        <v>59760706338</v>
       </c>
       <c r="K1156" t="n">
-        <v>57612007483</v>
+        <v>62305690457</v>
       </c>
     </row>
     <row r="1157">
       <c r="A1157" t="inlineStr">
         <is>
-          <t>1000.20.4</t>
+          <t>1000.10.4</t>
         </is>
       </c>
       <c r="B1157" t="n">
@@ -45452,31 +45446,25 @@
         <v>4500</v>
       </c>
       <c r="E1157" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F1157" t="n">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="G1157" t="n">
-        <v>3750.289861862383</v>
+        <v>1745.548800328407</v>
       </c>
       <c r="H1157" t="n">
-        <v>3676.25923851024</v>
-      </c>
-      <c r="I1157" t="n">
-        <v>3670.733398781877</v>
+        <v>1715.978513023062</v>
       </c>
       <c r="J1157" t="n">
-        <v>55598291229</v>
-      </c>
-      <c r="K1157" t="n">
-        <v>58759408779</v>
+        <v>59610645003</v>
       </c>
     </row>
     <row r="1158">
       <c r="A1158" t="inlineStr">
         <is>
-          <t>1000.20.4</t>
+          <t>1000.10.4</t>
         </is>
       </c>
       <c r="B1158" t="n">
@@ -45491,31 +45479,25 @@
         <v>4500</v>
       </c>
       <c r="E1158" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F1158" t="n">
-        <v>200</v>
+        <v>700</v>
       </c>
       <c r="G1158" t="n">
-        <v>3750.289861862383</v>
+        <v>1745.548800328407</v>
       </c>
       <c r="H1158" t="n">
-        <v>3662.58440372612</v>
-      </c>
-      <c r="I1158" t="n">
-        <v>3636.649673462108</v>
+        <v>1728.114763097489</v>
       </c>
       <c r="J1158" t="n">
-        <v>55666781684</v>
-      </c>
-      <c r="K1158" t="n">
-        <v>58678113114</v>
+        <v>59703415109</v>
       </c>
     </row>
     <row r="1159">
       <c r="A1159" t="inlineStr">
         <is>
-          <t>1000.20.4</t>
+          <t>1000.10.4</t>
         </is>
       </c>
       <c r="B1159" t="n">
@@ -45530,31 +45512,25 @@
         <v>4500</v>
       </c>
       <c r="E1159" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F1159" t="n">
-        <v>300</v>
+        <v>800</v>
       </c>
       <c r="G1159" t="n">
-        <v>3750.289861862383</v>
+        <v>1745.548800328407</v>
       </c>
       <c r="H1159" t="n">
-        <v>3640.786747235285</v>
-      </c>
-      <c r="I1159" t="n">
-        <v>3626.928613219296</v>
+        <v>1739.525746591372</v>
       </c>
       <c r="J1159" t="n">
-        <v>55705986427</v>
-      </c>
-      <c r="K1159" t="n">
-        <v>58360786268</v>
+        <v>59442222515</v>
       </c>
     </row>
     <row r="1160">
       <c r="A1160" t="inlineStr">
         <is>
-          <t>1000.20.4</t>
+          <t>1000.10.4</t>
         </is>
       </c>
       <c r="B1160" t="n">
@@ -45569,25 +45545,25 @@
         <v>4500</v>
       </c>
       <c r="E1160" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F1160" t="n">
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="G1160" t="n">
-        <v>3750.289861862383</v>
-      </c>
-      <c r="I1160" t="n">
-        <v>3649.085715187551</v>
-      </c>
-      <c r="K1160" t="n">
-        <v>58460871742</v>
+        <v>1745.548800328407</v>
+      </c>
+      <c r="H1160" t="n">
+        <v>1739.004081595807</v>
+      </c>
+      <c r="J1160" t="n">
+        <v>59477625709</v>
       </c>
     </row>
     <row r="1161">
       <c r="A1161" t="inlineStr">
         <is>
-          <t>1000.20.4</t>
+          <t>1000.10.4</t>
         </is>
       </c>
       <c r="B1161" t="n">
@@ -45602,25 +45578,25 @@
         <v>4500</v>
       </c>
       <c r="E1161" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F1161" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G1161" t="n">
-        <v>3750.289861862383</v>
-      </c>
-      <c r="I1161" t="n">
-        <v>3653.587321404143</v>
-      </c>
-      <c r="K1161" t="n">
-        <v>58573086462</v>
+        <v>1745.548800328407</v>
+      </c>
+      <c r="H1161" t="n">
+        <v>1745.048740707867</v>
+      </c>
+      <c r="J1161" t="n">
+        <v>59553159979</v>
       </c>
     </row>
     <row r="1162">
       <c r="A1162" t="inlineStr">
         <is>
-          <t>1000.30.1</t>
+          <t>1000.20.1</t>
         </is>
       </c>
       <c r="B1162" t="n">
@@ -45641,25 +45617,25 @@
         <v>100</v>
       </c>
       <c r="G1162" t="n">
-        <v>7979.543044930953</v>
+        <v>3708.541021396037</v>
       </c>
       <c r="H1162" t="n">
-        <v>7909.942853594655</v>
+        <v>3711.484141374198</v>
       </c>
       <c r="I1162" t="n">
-        <v>7903.870424714833</v>
+        <v>3709.684088929843</v>
       </c>
       <c r="J1162" t="n">
-        <v>75322972139</v>
+        <v>54539220721</v>
       </c>
       <c r="K1162" t="n">
-        <v>80290385520</v>
+        <v>57058097271</v>
       </c>
     </row>
     <row r="1163">
       <c r="A1163" t="inlineStr">
         <is>
-          <t>1000.30.1</t>
+          <t>1000.20.1</t>
         </is>
       </c>
       <c r="B1163" t="n">
@@ -45680,25 +45656,25 @@
         <v>200</v>
       </c>
       <c r="G1163" t="n">
-        <v>7979.543044930953</v>
+        <v>3708.541021396037</v>
       </c>
       <c r="H1163" t="n">
-        <v>7933.369653078021</v>
+        <v>3717.075646092836</v>
       </c>
       <c r="I1163" t="n">
-        <v>7887.053929253325</v>
+        <v>3712.684249728848</v>
       </c>
       <c r="J1163" t="n">
-        <v>75779392870</v>
+        <v>54746244345</v>
       </c>
       <c r="K1163" t="n">
-        <v>80350357454</v>
+        <v>57502335211</v>
       </c>
     </row>
     <row r="1164">
       <c r="A1164" t="inlineStr">
         <is>
-          <t>1000.30.1</t>
+          <t>1000.20.1</t>
         </is>
       </c>
       <c r="B1164" t="n">
@@ -45719,25 +45695,25 @@
         <v>300</v>
       </c>
       <c r="G1164" t="n">
-        <v>7979.543044930953</v>
+        <v>3708.541021396037</v>
       </c>
       <c r="H1164" t="n">
-        <v>7938.674740845327</v>
+        <v>3709.542619220546</v>
       </c>
       <c r="I1164" t="n">
-        <v>7907.193593195034</v>
+        <v>3710.003790441718</v>
       </c>
       <c r="J1164" t="n">
-        <v>75826655517</v>
+        <v>54542720537</v>
       </c>
       <c r="K1164" t="n">
-        <v>80336749536</v>
+        <v>57084344927</v>
       </c>
     </row>
     <row r="1165">
       <c r="A1165" t="inlineStr">
         <is>
-          <t>1000.30.1</t>
+          <t>1000.20.1</t>
         </is>
       </c>
       <c r="B1165" t="n">
@@ -45758,19 +45734,25 @@
         <v>400</v>
       </c>
       <c r="G1165" t="n">
-        <v>7979.543044930953</v>
+        <v>3708.541021396037</v>
+      </c>
+      <c r="H1165" t="n">
+        <v>3715.854849154871</v>
       </c>
       <c r="I1165" t="n">
-        <v>7928.849627264417</v>
+        <v>3715.817786494159</v>
+      </c>
+      <c r="J1165" t="n">
+        <v>54782026539</v>
       </c>
       <c r="K1165" t="n">
-        <v>80058172429</v>
+        <v>57407086972</v>
       </c>
     </row>
     <row r="1166">
       <c r="A1166" t="inlineStr">
         <is>
-          <t>1000.30.1</t>
+          <t>1000.20.1</t>
         </is>
       </c>
       <c r="B1166" t="n">
@@ -45791,19 +45773,25 @@
         <v>500</v>
       </c>
       <c r="G1166" t="n">
-        <v>7979.543044930953</v>
+        <v>3708.541021396037</v>
+      </c>
+      <c r="H1166" t="n">
+        <v>3724.648872747662</v>
       </c>
       <c r="I1166" t="n">
-        <v>7918.811182482041</v>
+        <v>3724.648872747662</v>
+      </c>
+      <c r="J1166" t="n">
+        <v>54637947401</v>
       </c>
       <c r="K1166" t="n">
-        <v>80136357169</v>
+        <v>57367898275</v>
       </c>
     </row>
     <row r="1167">
       <c r="A1167" t="inlineStr">
         <is>
-          <t>1000.30.2</t>
+          <t>1000.20.1</t>
         </is>
       </c>
       <c r="B1167" t="n">
@@ -45818,31 +45806,25 @@
         <v>4500</v>
       </c>
       <c r="E1167" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F1167" t="n">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="G1167" t="n">
-        <v>7973.009423005142</v>
+        <v>3708.541021396037</v>
       </c>
       <c r="H1167" t="n">
-        <v>7955.478963396214</v>
-      </c>
-      <c r="I1167" t="n">
-        <v>7944.300020434308</v>
+        <v>3746.459096600642</v>
       </c>
       <c r="J1167" t="n">
-        <v>75463252430</v>
-      </c>
-      <c r="K1167" t="n">
-        <v>79665719147</v>
+        <v>54662929032</v>
       </c>
     </row>
     <row r="1168">
       <c r="A1168" t="inlineStr">
         <is>
-          <t>1000.30.2</t>
+          <t>1000.20.1</t>
         </is>
       </c>
       <c r="B1168" t="n">
@@ -45857,31 +45839,25 @@
         <v>4500</v>
       </c>
       <c r="E1168" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F1168" t="n">
-        <v>200</v>
+        <v>700</v>
       </c>
       <c r="G1168" t="n">
-        <v>7973.009423005142</v>
+        <v>3708.541021396037</v>
       </c>
       <c r="H1168" t="n">
-        <v>7985.667796737807</v>
-      </c>
-      <c r="I1168" t="n">
-        <v>7950.033926181859</v>
+        <v>3712.551616640903</v>
       </c>
       <c r="J1168" t="n">
-        <v>75499709671</v>
-      </c>
-      <c r="K1168" t="n">
-        <v>79559486593</v>
+        <v>54809094607</v>
       </c>
     </row>
     <row r="1169">
       <c r="A1169" t="inlineStr">
         <is>
-          <t>1000.30.2</t>
+          <t>1000.20.1</t>
         </is>
       </c>
       <c r="B1169" t="n">
@@ -45896,31 +45872,25 @@
         <v>4500</v>
       </c>
       <c r="E1169" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F1169" t="n">
-        <v>300</v>
+        <v>800</v>
       </c>
       <c r="G1169" t="n">
-        <v>7973.009423005142</v>
+        <v>3708.541021396037</v>
       </c>
       <c r="H1169" t="n">
-        <v>7971.863557246797</v>
-      </c>
-      <c r="I1169" t="n">
-        <v>7945.713457379617</v>
+        <v>3724.489476987844</v>
       </c>
       <c r="J1169" t="n">
-        <v>75291910014</v>
-      </c>
-      <c r="K1169" t="n">
-        <v>79646776106</v>
+        <v>54759404675</v>
       </c>
     </row>
     <row r="1170">
       <c r="A1170" t="inlineStr">
         <is>
-          <t>1000.30.2</t>
+          <t>1000.20.1</t>
         </is>
       </c>
       <c r="B1170" t="n">
@@ -45935,25 +45905,25 @@
         <v>4500</v>
       </c>
       <c r="E1170" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F1170" t="n">
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="G1170" t="n">
-        <v>7973.009423005142</v>
-      </c>
-      <c r="I1170" t="n">
-        <v>7959.459092132034</v>
-      </c>
-      <c r="K1170" t="n">
-        <v>79191579668</v>
+        <v>3708.541021396037</v>
+      </c>
+      <c r="H1170" t="n">
+        <v>3722.164180205413</v>
+      </c>
+      <c r="J1170" t="n">
+        <v>54598042516</v>
       </c>
     </row>
     <row r="1171">
       <c r="A1171" t="inlineStr">
         <is>
-          <t>1000.30.2</t>
+          <t>1000.20.1</t>
         </is>
       </c>
       <c r="B1171" t="n">
@@ -45968,25 +45938,25 @@
         <v>4500</v>
       </c>
       <c r="E1171" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F1171" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G1171" t="n">
-        <v>7973.009423005142</v>
-      </c>
-      <c r="I1171" t="n">
-        <v>7970.03120460759</v>
-      </c>
-      <c r="K1171" t="n">
-        <v>80012508520</v>
+        <v>3708.541021396037</v>
+      </c>
+      <c r="H1171" t="n">
+        <v>3733.340975642415</v>
+      </c>
+      <c r="J1171" t="n">
+        <v>54951260017</v>
       </c>
     </row>
     <row r="1172">
       <c r="A1172" t="inlineStr">
         <is>
-          <t>1000.30.3</t>
+          <t>1000.20.2</t>
         </is>
       </c>
       <c r="B1172" t="n">
@@ -46007,25 +45977,25 @@
         <v>100</v>
       </c>
       <c r="G1172" t="n">
-        <v>7977.814850915422</v>
+        <v>3768.103517429845</v>
       </c>
       <c r="H1172" t="n">
-        <v>7912.800374705674</v>
+        <v>3718.334914449701</v>
       </c>
       <c r="I1172" t="n">
-        <v>7920.722535902631</v>
+        <v>3707.205779416522</v>
       </c>
       <c r="J1172" t="n">
-        <v>75526679782</v>
+        <v>54522257604</v>
       </c>
       <c r="K1172" t="n">
-        <v>79864223403</v>
+        <v>56748923914</v>
       </c>
     </row>
     <row r="1173">
       <c r="A1173" t="inlineStr">
         <is>
-          <t>1000.30.3</t>
+          <t>1000.20.2</t>
         </is>
       </c>
       <c r="B1173" t="n">
@@ -46046,25 +46016,25 @@
         <v>200</v>
       </c>
       <c r="G1173" t="n">
-        <v>7977.814850915422</v>
+        <v>3768.103517429845</v>
       </c>
       <c r="H1173" t="n">
-        <v>7920.286934325561</v>
+        <v>3712.59434092089</v>
       </c>
       <c r="I1173" t="n">
-        <v>7876.350396623391</v>
+        <v>3688.571250633831</v>
       </c>
       <c r="J1173" t="n">
-        <v>75239934410</v>
+        <v>54713477727</v>
       </c>
       <c r="K1173" t="n">
-        <v>79854507057</v>
+        <v>57558889306</v>
       </c>
     </row>
     <row r="1174">
       <c r="A1174" t="inlineStr">
         <is>
-          <t>1000.30.3</t>
+          <t>1000.20.2</t>
         </is>
       </c>
       <c r="B1174" t="n">
@@ -46085,25 +46055,25 @@
         <v>300</v>
       </c>
       <c r="G1174" t="n">
-        <v>7977.814850915422</v>
+        <v>3768.103517429845</v>
       </c>
       <c r="H1174" t="n">
-        <v>7913.559085252405</v>
+        <v>3730.776752188581</v>
       </c>
       <c r="I1174" t="n">
-        <v>7860.33109598247</v>
+        <v>3725.00272664874</v>
       </c>
       <c r="J1174" t="n">
-        <v>75154106633</v>
+        <v>54778015958</v>
       </c>
       <c r="K1174" t="n">
-        <v>79559590331</v>
+        <v>57374818287</v>
       </c>
     </row>
     <row r="1175">
       <c r="A1175" t="inlineStr">
         <is>
-          <t>1000.30.3</t>
+          <t>1000.20.2</t>
         </is>
       </c>
       <c r="B1175" t="n">
@@ -46124,19 +46094,25 @@
         <v>400</v>
       </c>
       <c r="G1175" t="n">
-        <v>7977.814850915422</v>
+        <v>3768.103517429845</v>
+      </c>
+      <c r="H1175" t="n">
+        <v>3724.21727260637</v>
       </c>
       <c r="I1175" t="n">
-        <v>7920.365306495831</v>
+        <v>3731.317629012444</v>
+      </c>
+      <c r="J1175" t="n">
+        <v>54955670135</v>
       </c>
       <c r="K1175" t="n">
-        <v>79839038862</v>
+        <v>57923996919</v>
       </c>
     </row>
     <row r="1176">
       <c r="A1176" t="inlineStr">
         <is>
-          <t>1000.30.3</t>
+          <t>1000.20.2</t>
         </is>
       </c>
       <c r="B1176" t="n">
@@ -46157,19 +46133,25 @@
         <v>500</v>
       </c>
       <c r="G1176" t="n">
-        <v>7977.814850915422</v>
+        <v>3768.103517429845</v>
+      </c>
+      <c r="H1176" t="n">
+        <v>3693.967339916833</v>
       </c>
       <c r="I1176" t="n">
-        <v>7864.197629346444</v>
+        <v>3698.256619021398</v>
+      </c>
+      <c r="J1176" t="n">
+        <v>54825219895</v>
       </c>
       <c r="K1176" t="n">
-        <v>79809132821</v>
+        <v>57292622262</v>
       </c>
     </row>
     <row r="1177">
       <c r="A1177" t="inlineStr">
         <is>
-          <t>1000.30.4</t>
+          <t>1000.20.2</t>
         </is>
       </c>
       <c r="B1177" t="n">
@@ -46184,31 +46166,25 @@
         <v>4500</v>
       </c>
       <c r="E1177" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F1177" t="n">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="G1177" t="n">
-        <v>7964.046250435393</v>
+        <v>3768.103517429845</v>
       </c>
       <c r="H1177" t="n">
-        <v>7954.622756722229</v>
-      </c>
-      <c r="I1177" t="n">
-        <v>7937.350316798198</v>
+        <v>3700.833521391454</v>
       </c>
       <c r="J1177" t="n">
-        <v>76298686901</v>
-      </c>
-      <c r="K1177" t="n">
-        <v>80345994552</v>
+        <v>54676570942</v>
       </c>
     </row>
     <row r="1178">
       <c r="A1178" t="inlineStr">
         <is>
-          <t>1000.30.4</t>
+          <t>1000.20.2</t>
         </is>
       </c>
       <c r="B1178" t="n">
@@ -46223,31 +46199,25 @@
         <v>4500</v>
       </c>
       <c r="E1178" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F1178" t="n">
-        <v>200</v>
+        <v>700</v>
       </c>
       <c r="G1178" t="n">
-        <v>7964.046250435393</v>
+        <v>3768.103517429845</v>
       </c>
       <c r="H1178" t="n">
-        <v>7944.878378597256</v>
-      </c>
-      <c r="I1178" t="n">
-        <v>7945.437917149456</v>
+        <v>3737.531688329461</v>
       </c>
       <c r="J1178" t="n">
-        <v>76143958723</v>
-      </c>
-      <c r="K1178" t="n">
-        <v>80072300346</v>
+        <v>54630006030</v>
       </c>
     </row>
     <row r="1179">
       <c r="A1179" t="inlineStr">
         <is>
-          <t>1000.30.4</t>
+          <t>1000.20.2</t>
         </is>
       </c>
       <c r="B1179" t="n">
@@ -46262,31 +46232,25 @@
         <v>4500</v>
       </c>
       <c r="E1179" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F1179" t="n">
-        <v>300</v>
+        <v>800</v>
       </c>
       <c r="G1179" t="n">
-        <v>7964.046250435393</v>
+        <v>3768.103517429845</v>
       </c>
       <c r="H1179" t="n">
-        <v>7908.149940826446</v>
-      </c>
-      <c r="I1179" t="n">
-        <v>7924.585067946708</v>
+        <v>3701.454862113157</v>
       </c>
       <c r="J1179" t="n">
-        <v>76310818841</v>
-      </c>
-      <c r="K1179" t="n">
-        <v>80329220533</v>
+        <v>55075525454</v>
       </c>
     </row>
     <row r="1180">
       <c r="A1180" t="inlineStr">
         <is>
-          <t>1000.30.4</t>
+          <t>1000.20.2</t>
         </is>
       </c>
       <c r="B1180" t="n">
@@ -46301,25 +46265,25 @@
         <v>4500</v>
       </c>
       <c r="E1180" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F1180" t="n">
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="G1180" t="n">
-        <v>7964.046250435393</v>
-      </c>
-      <c r="I1180" t="n">
-        <v>7929.577010942594</v>
-      </c>
-      <c r="K1180" t="n">
-        <v>79863930995</v>
+        <v>3768.103517429845</v>
+      </c>
+      <c r="H1180" t="n">
+        <v>3701.038233464449</v>
+      </c>
+      <c r="J1180" t="n">
+        <v>54950125042</v>
       </c>
     </row>
     <row r="1181">
       <c r="A1181" t="inlineStr">
         <is>
-          <t>1000.30.4</t>
+          <t>1000.20.2</t>
         </is>
       </c>
       <c r="B1181" t="n">
@@ -46334,25 +46298,25 @@
         <v>4500</v>
       </c>
       <c r="E1181" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F1181" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G1181" t="n">
-        <v>7964.046250435393</v>
-      </c>
-      <c r="I1181" t="n">
-        <v>7907.056895020358</v>
-      </c>
-      <c r="K1181" t="n">
-        <v>80221553843</v>
+        <v>3768.103517429845</v>
+      </c>
+      <c r="H1181" t="n">
+        <v>3715.729199532919</v>
+      </c>
+      <c r="J1181" t="n">
+        <v>54303352544</v>
       </c>
     </row>
     <row r="1182">
       <c r="A1182" t="inlineStr">
         <is>
-          <t>1000.40.1</t>
+          <t>1000.20.3</t>
         </is>
       </c>
       <c r="B1182" t="n">
@@ -46373,25 +46337,25 @@
         <v>100</v>
       </c>
       <c r="G1182" t="n">
-        <v>14005.02994874948</v>
+        <v>3734.724211492563</v>
       </c>
       <c r="H1182" t="n">
-        <v>13804.65911026816</v>
+        <v>3675.718557688236</v>
       </c>
       <c r="I1182" t="n">
-        <v>13727.06070999957</v>
+        <v>3679.378142308556</v>
       </c>
       <c r="J1182" t="n">
-        <v>85252367167</v>
+        <v>55234934660</v>
       </c>
       <c r="K1182" t="n">
-        <v>87948448001</v>
+        <v>57888578439</v>
       </c>
     </row>
     <row r="1183">
       <c r="A1183" t="inlineStr">
         <is>
-          <t>1000.40.1</t>
+          <t>1000.20.3</t>
         </is>
       </c>
       <c r="B1183" t="n">
@@ -46412,25 +46376,25 @@
         <v>200</v>
       </c>
       <c r="G1183" t="n">
-        <v>14005.02994874948</v>
+        <v>3734.724211492563</v>
       </c>
       <c r="H1183" t="n">
-        <v>13703.5761313689</v>
+        <v>3671.040088594132</v>
       </c>
       <c r="I1183" t="n">
-        <v>13678.77539809002</v>
+        <v>3661.716562358774</v>
       </c>
       <c r="J1183" t="n">
-        <v>85000059396</v>
+        <v>55008199465</v>
       </c>
       <c r="K1183" t="n">
-        <v>88387691033</v>
+        <v>58027715698</v>
       </c>
     </row>
     <row r="1184">
       <c r="A1184" t="inlineStr">
         <is>
-          <t>1000.40.1</t>
+          <t>1000.20.3</t>
         </is>
       </c>
       <c r="B1184" t="n">
@@ -46451,25 +46415,25 @@
         <v>300</v>
       </c>
       <c r="G1184" t="n">
-        <v>14005.02994874948</v>
+        <v>3734.724211492563</v>
       </c>
       <c r="H1184" t="n">
-        <v>13829.70485039924</v>
+        <v>3679.658407988477</v>
       </c>
       <c r="I1184" t="n">
-        <v>13707.46434839891</v>
+        <v>3666.047778478794</v>
       </c>
       <c r="J1184" t="n">
-        <v>84913861591</v>
+        <v>54859740947</v>
       </c>
       <c r="K1184" t="n">
-        <v>88130654686</v>
+        <v>57560856429</v>
       </c>
     </row>
     <row r="1185">
       <c r="A1185" t="inlineStr">
         <is>
-          <t>1000.40.1</t>
+          <t>1000.20.3</t>
         </is>
       </c>
       <c r="B1185" t="n">
@@ -46490,19 +46454,25 @@
         <v>400</v>
       </c>
       <c r="G1185" t="n">
-        <v>14005.02994874948</v>
+        <v>3734.724211492563</v>
+      </c>
+      <c r="H1185" t="n">
+        <v>3689.419253356074</v>
       </c>
       <c r="I1185" t="n">
-        <v>13740.21554885748</v>
+        <v>3671.922246025872</v>
+      </c>
+      <c r="J1185" t="n">
+        <v>54882210459</v>
       </c>
       <c r="K1185" t="n">
-        <v>88297144687</v>
+        <v>57868215020</v>
       </c>
     </row>
     <row r="1186">
       <c r="A1186" t="inlineStr">
         <is>
-          <t>1000.40.1</t>
+          <t>1000.20.3</t>
         </is>
       </c>
       <c r="B1186" t="n">
@@ -46523,19 +46493,25 @@
         <v>500</v>
       </c>
       <c r="G1186" t="n">
-        <v>14005.02994874948</v>
+        <v>3734.724211492563</v>
+      </c>
+      <c r="H1186" t="n">
+        <v>3707.49988556537</v>
       </c>
       <c r="I1186" t="n">
-        <v>13666.85921821061</v>
+        <v>3692.032536338156</v>
+      </c>
+      <c r="J1186" t="n">
+        <v>54852225100</v>
       </c>
       <c r="K1186" t="n">
-        <v>88392609632</v>
+        <v>57612007483</v>
       </c>
     </row>
     <row r="1187">
       <c r="A1187" t="inlineStr">
         <is>
-          <t>1000.40.2</t>
+          <t>1000.20.3</t>
         </is>
       </c>
       <c r="B1187" t="n">
@@ -46550,31 +46526,25 @@
         <v>4500</v>
       </c>
       <c r="E1187" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F1187" t="n">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="G1187" t="n">
-        <v>14118.04105210099</v>
+        <v>3734.724211492563</v>
       </c>
       <c r="H1187" t="n">
-        <v>13953.57733794516</v>
-      </c>
-      <c r="I1187" t="n">
-        <v>13931.39017551439</v>
+        <v>3675.950951253969</v>
       </c>
       <c r="J1187" t="n">
-        <v>84476830074</v>
-      </c>
-      <c r="K1187" t="n">
-        <v>88463191445</v>
+        <v>55095800349</v>
       </c>
     </row>
     <row r="1188">
       <c r="A1188" t="inlineStr">
         <is>
-          <t>1000.40.2</t>
+          <t>1000.20.3</t>
         </is>
       </c>
       <c r="B1188" t="n">
@@ -46589,31 +46559,25 @@
         <v>4500</v>
       </c>
       <c r="E1188" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F1188" t="n">
-        <v>200</v>
+        <v>700</v>
       </c>
       <c r="G1188" t="n">
-        <v>14118.04105210099</v>
+        <v>3734.724211492563</v>
       </c>
       <c r="H1188" t="n">
-        <v>13879.86269944144</v>
-      </c>
-      <c r="I1188" t="n">
-        <v>13850.72930858321</v>
+        <v>3681.728201160339</v>
       </c>
       <c r="J1188" t="n">
-        <v>84567750703</v>
-      </c>
-      <c r="K1188" t="n">
-        <v>88374159109</v>
+        <v>55476519613</v>
       </c>
     </row>
     <row r="1189">
       <c r="A1189" t="inlineStr">
         <is>
-          <t>1000.40.2</t>
+          <t>1000.20.3</t>
         </is>
       </c>
       <c r="B1189" t="n">
@@ -46628,31 +46592,25 @@
         <v>4500</v>
       </c>
       <c r="E1189" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F1189" t="n">
-        <v>300</v>
+        <v>800</v>
       </c>
       <c r="G1189" t="n">
-        <v>14118.04105210099</v>
+        <v>3734.724211492563</v>
       </c>
       <c r="H1189" t="n">
-        <v>13960.02681644472</v>
-      </c>
-      <c r="I1189" t="n">
-        <v>13917.82365179558</v>
+        <v>3699.34610647119</v>
       </c>
       <c r="J1189" t="n">
-        <v>84895471386</v>
-      </c>
-      <c r="K1189" t="n">
-        <v>88267450156</v>
+        <v>55168729495</v>
       </c>
     </row>
     <row r="1190">
       <c r="A1190" t="inlineStr">
         <is>
-          <t>1000.40.2</t>
+          <t>1000.20.3</t>
         </is>
       </c>
       <c r="B1190" t="n">
@@ -46667,25 +46625,25 @@
         <v>4500</v>
       </c>
       <c r="E1190" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F1190" t="n">
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="G1190" t="n">
-        <v>14118.04105210099</v>
-      </c>
-      <c r="I1190" t="n">
-        <v>13860.35154425662</v>
-      </c>
-      <c r="K1190" t="n">
-        <v>88312094525</v>
+        <v>3734.724211492563</v>
+      </c>
+      <c r="H1190" t="n">
+        <v>3686.45567627628</v>
+      </c>
+      <c r="J1190" t="n">
+        <v>55151096875</v>
       </c>
     </row>
     <row r="1191">
       <c r="A1191" t="inlineStr">
         <is>
-          <t>1000.40.2</t>
+          <t>1000.20.3</t>
         </is>
       </c>
       <c r="B1191" t="n">
@@ -46700,25 +46658,25 @@
         <v>4500</v>
       </c>
       <c r="E1191" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F1191" t="n">
-        <v>500</v>
+        <v>1000</v>
       </c>
       <c r="G1191" t="n">
-        <v>14118.04105210099</v>
-      </c>
-      <c r="I1191" t="n">
-        <v>13816.65492916855</v>
-      </c>
-      <c r="K1191" t="n">
-        <v>88256861778</v>
+        <v>3734.724211492563</v>
+      </c>
+      <c r="H1191" t="n">
+        <v>3712.571582138261</v>
+      </c>
+      <c r="J1191" t="n">
+        <v>55097006370</v>
       </c>
     </row>
     <row r="1192">
       <c r="A1192" t="inlineStr">
         <is>
-          <t>1000.40.3</t>
+          <t>1000.20.4</t>
         </is>
       </c>
       <c r="B1192" t="n">
@@ -46739,25 +46697,25 @@
         <v>100</v>
       </c>
       <c r="G1192" t="n">
-        <v>14052.70747046845</v>
+        <v>3750.289861862383</v>
       </c>
       <c r="H1192" t="n">
-        <v>13928.43424030587</v>
+        <v>3676.25923851024</v>
       </c>
       <c r="I1192" t="n">
-        <v>13866.49181471369</v>
+        <v>3670.733398781877</v>
       </c>
       <c r="J1192" t="n">
-        <v>84955360440</v>
+        <v>55598291229</v>
       </c>
       <c r="K1192" t="n">
-        <v>88491758334</v>
+        <v>58759408779</v>
       </c>
     </row>
     <row r="1193">
       <c r="A1193" t="inlineStr">
         <is>
-          <t>1000.40.3</t>
+          <t>1000.20.4</t>
         </is>
       </c>
       <c r="B1193" t="n">
@@ -46778,25 +46736,25 @@
         <v>200</v>
       </c>
       <c r="G1193" t="n">
-        <v>14052.70747046845</v>
+        <v>3750.289861862383</v>
       </c>
       <c r="H1193" t="n">
-        <v>14025.13225262927</v>
+        <v>3662.58440372612</v>
       </c>
       <c r="I1193" t="n">
-        <v>13992.15523571734</v>
+        <v>3636.649673462108</v>
       </c>
       <c r="J1193" t="n">
-        <v>84845024911</v>
+        <v>55666781684</v>
       </c>
       <c r="K1193" t="n">
-        <v>88258794676</v>
+        <v>58678113114</v>
       </c>
     </row>
     <row r="1194">
       <c r="A1194" t="inlineStr">
         <is>
-          <t>1000.40.3</t>
+          <t>1000.20.4</t>
         </is>
       </c>
       <c r="B1194" t="n">
@@ -46817,25 +46775,25 @@
         <v>300</v>
       </c>
       <c r="G1194" t="n">
-        <v>14052.70747046845</v>
+        <v>3750.289861862383</v>
       </c>
       <c r="H1194" t="n">
-        <v>13988.34944155203</v>
+        <v>3640.786747235285</v>
       </c>
       <c r="I1194" t="n">
-        <v>13922.58586497711</v>
+        <v>3626.928613219296</v>
       </c>
       <c r="J1194" t="n">
-        <v>85041302241</v>
+        <v>55705986427</v>
       </c>
       <c r="K1194" t="n">
-        <v>88291746606</v>
+        <v>58360786268</v>
       </c>
     </row>
     <row r="1195">
       <c r="A1195" t="inlineStr">
         <is>
-          <t>1000.40.3</t>
+          <t>1000.20.4</t>
         </is>
       </c>
       <c r="B1195" t="n">
@@ -46856,19 +46814,25 @@
         <v>400</v>
       </c>
       <c r="G1195" t="n">
-        <v>14052.70747046845</v>
+        <v>3750.289861862383</v>
+      </c>
+      <c r="H1195" t="n">
+        <v>3658.158045349088</v>
       </c>
       <c r="I1195" t="n">
-        <v>13985.74834269132</v>
+        <v>3649.085715187551</v>
+      </c>
+      <c r="J1195" t="n">
+        <v>55781519621</v>
       </c>
       <c r="K1195" t="n">
-        <v>88070207994</v>
+        <v>58460871742</v>
       </c>
     </row>
     <row r="1196">
       <c r="A1196" t="inlineStr">
         <is>
-          <t>1000.40.3</t>
+          <t>1000.20.4</t>
         </is>
       </c>
       <c r="B1196" t="n">
@@ -46889,19 +46853,25 @@
         <v>500</v>
       </c>
       <c r="G1196" t="n">
-        <v>14052.70747046845</v>
+        <v>3750.289861862383</v>
+      </c>
+      <c r="H1196" t="n">
+        <v>3671.38826635242</v>
       </c>
       <c r="I1196" t="n">
-        <v>13920.36568946934</v>
+        <v>3653.587321404143</v>
+      </c>
+      <c r="J1196" t="n">
+        <v>55710337214</v>
       </c>
       <c r="K1196" t="n">
-        <v>88382124558</v>
+        <v>58573086462</v>
       </c>
     </row>
     <row r="1197">
       <c r="A1197" t="inlineStr">
         <is>
-          <t>1000.40.4</t>
+          <t>1000.20.4</t>
         </is>
       </c>
       <c r="B1197" t="n">
@@ -46916,31 +46886,25 @@
         <v>4500</v>
       </c>
       <c r="E1197" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F1197" t="n">
-        <v>100</v>
+        <v>600</v>
       </c>
       <c r="G1197" t="n">
-        <v>14047.58679159633</v>
+        <v>3750.289861862383</v>
       </c>
       <c r="H1197" t="n">
-        <v>13855.13481452877</v>
-      </c>
-      <c r="I1197" t="n">
-        <v>13769.51168139956</v>
+        <v>3671.789267733619</v>
       </c>
       <c r="J1197" t="n">
-        <v>84108180671</v>
-      </c>
-      <c r="K1197" t="n">
-        <v>88169613935</v>
+        <v>55592915338</v>
       </c>
     </row>
     <row r="1198">
       <c r="A1198" t="inlineStr">
         <is>
-          <t>1000.40.4</t>
+          <t>1000.20.4</t>
         </is>
       </c>
       <c r="B1198" t="n">
@@ -46955,31 +46919,25 @@
         <v>4500</v>
       </c>
       <c r="E1198" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="F1198" t="n">
-        <v>200</v>
+        <v>700</v>
       </c>
       <c r="G1198" t="n">
-        <v>14047.58679159633</v>
+        <v>3750.289861862383</v>
       </c>
       <c r="H1198" t="n">
-        <v>13808.05311567009</v>
-      </c>
-      <c r="I1198" t="n">
-        <v>13792.0484138216</v>
+        <v>3661.915773637411</v>
       </c>
       <c r="J1198" t="n">
-        <v>83932164076</v>
-      </c>
-      <c r="K1198" t="n">
-        <v>87849710144</v>
+        <v>55832302836</v>
       </c>
     </row>
     <row r="1199">
       <c r="A1199" t="inlineStr">
         <is>
-          <t>1000.40.4</t>
+          <t>1000.20.4</t>
         </is>
       </c>
       <c r="B1199" t="n">
@@ -46994,31 +46952,25 @@
         <v>4500</v>
       </c>
       <c r="E1199" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="F1199" t="n">
-        <v>300</v>
+        <v>800</v>
       </c>
       <c r="G1199" t="n">
-        <v>14047.58679159633</v>
+        <v>3750.289861862383</v>
       </c>
       <c r="H1199" t="n">
-        <v>13788.06577326823</v>
-      </c>
-      <c r="I1199" t="n">
-        <v>13833.52844773018</v>
+        <v>3669.840810726894</v>
       </c>
       <c r="J1199" t="n">
-        <v>84099856887</v>
-      </c>
-      <c r="K1199" t="n">
-        <v>88168171393</v>
+        <v>55777809317</v>
       </c>
     </row>
     <row r="1200">
       <c r="A1200" t="inlineStr">
         <is>
-          <t>1000.40.4</t>
+          <t>1000.20.4</t>
         </is>
       </c>
       <c r="B1200" t="n">
@@ -47033,25 +46985,25 @@
         <v>4500</v>
       </c>
       <c r="E1200" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="F1200" t="n">
-        <v>400</v>
+        <v>900</v>
       </c>
       <c r="G1200" t="n">
-        <v>14047.58679159633</v>
-      </c>
-      <c r="I1200" t="n">
-        <v>13774.94086040058</v>
-      </c>
-      <c r="K1200" t="n">
-        <v>87919633198</v>
+        <v>3750.289861862383</v>
+      </c>
+      <c r="H1200" t="n">
+        <v>3693.94371769767</v>
+      </c>
+      <c r="J1200" t="n">
+        <v>56129453598</v>
       </c>
     </row>
     <row r="1201">
       <c r="A1201" t="inlineStr">
         <is>
-          <t>1000.40.4</t>
+          <t>1000.20.4</t>
         </is>
       </c>
       <c r="B1201" t="n">
@@ -47066,18 +47018,1980 @@
         <v>4500</v>
       </c>
       <c r="E1201" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1201" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G1201" t="n">
+        <v>3750.289861862383</v>
+      </c>
+      <c r="H1201" t="n">
+        <v>3634.221390650036</v>
+      </c>
+      <c r="J1201" t="n">
+        <v>55857258078</v>
+      </c>
+    </row>
+    <row r="1202">
+      <c r="A1202" t="inlineStr">
+        <is>
+          <t>1000.30.1</t>
+        </is>
+      </c>
+      <c r="B1202" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1202" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1202" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1202" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1202" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1202" t="n">
+        <v>7979.543044930953</v>
+      </c>
+      <c r="H1202" t="n">
+        <v>7909.942853594655</v>
+      </c>
+      <c r="I1202" t="n">
+        <v>7903.870424714833</v>
+      </c>
+      <c r="J1202" t="n">
+        <v>75322972139</v>
+      </c>
+      <c r="K1202" t="n">
+        <v>80290385520</v>
+      </c>
+    </row>
+    <row r="1203">
+      <c r="A1203" t="inlineStr">
+        <is>
+          <t>1000.30.1</t>
+        </is>
+      </c>
+      <c r="B1203" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1203" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1203" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1203" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1203" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1203" t="n">
+        <v>7979.543044930953</v>
+      </c>
+      <c r="H1203" t="n">
+        <v>7933.369653078021</v>
+      </c>
+      <c r="I1203" t="n">
+        <v>7887.053929253325</v>
+      </c>
+      <c r="J1203" t="n">
+        <v>75779392870</v>
+      </c>
+      <c r="K1203" t="n">
+        <v>80350357454</v>
+      </c>
+    </row>
+    <row r="1204">
+      <c r="A1204" t="inlineStr">
+        <is>
+          <t>1000.30.1</t>
+        </is>
+      </c>
+      <c r="B1204" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1204" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1204" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1204" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1204" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1204" t="n">
+        <v>7979.543044930953</v>
+      </c>
+      <c r="H1204" t="n">
+        <v>7938.674740845327</v>
+      </c>
+      <c r="I1204" t="n">
+        <v>7907.193593195034</v>
+      </c>
+      <c r="J1204" t="n">
+        <v>75826655517</v>
+      </c>
+      <c r="K1204" t="n">
+        <v>80336749536</v>
+      </c>
+    </row>
+    <row r="1205">
+      <c r="A1205" t="inlineStr">
+        <is>
+          <t>1000.30.1</t>
+        </is>
+      </c>
+      <c r="B1205" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1205" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1205" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1205" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1205" t="n">
+        <v>400</v>
+      </c>
+      <c r="G1205" t="n">
+        <v>7979.543044930953</v>
+      </c>
+      <c r="H1205" t="n">
+        <v>7907.676600882356</v>
+      </c>
+      <c r="I1205" t="n">
+        <v>7928.849627264417</v>
+      </c>
+      <c r="J1205" t="n">
+        <v>75784612237</v>
+      </c>
+      <c r="K1205" t="n">
+        <v>80058172429</v>
+      </c>
+    </row>
+    <row r="1206">
+      <c r="A1206" t="inlineStr">
+        <is>
+          <t>1000.30.1</t>
+        </is>
+      </c>
+      <c r="B1206" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1206" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1206" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1206" t="n">
         <v>5</v>
       </c>
-      <c r="F1201" t="n">
+      <c r="F1206" t="n">
         <v>500</v>
       </c>
-      <c r="G1201" t="n">
+      <c r="G1206" t="n">
+        <v>7979.543044930953</v>
+      </c>
+      <c r="H1206" t="n">
+        <v>7919.890889033499</v>
+      </c>
+      <c r="I1206" t="n">
+        <v>7918.811182482041</v>
+      </c>
+      <c r="J1206" t="n">
+        <v>75867899125</v>
+      </c>
+      <c r="K1206" t="n">
+        <v>80136357169</v>
+      </c>
+    </row>
+    <row r="1207">
+      <c r="A1207" t="inlineStr">
+        <is>
+          <t>1000.30.1</t>
+        </is>
+      </c>
+      <c r="B1207" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1207" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1207" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1207" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1207" t="n">
+        <v>600</v>
+      </c>
+      <c r="G1207" t="n">
+        <v>7979.543044930953</v>
+      </c>
+      <c r="H1207" t="n">
+        <v>7950.820550352748</v>
+      </c>
+      <c r="J1207" t="n">
+        <v>75912438625</v>
+      </c>
+    </row>
+    <row r="1208">
+      <c r="A1208" t="inlineStr">
+        <is>
+          <t>1000.30.1</t>
+        </is>
+      </c>
+      <c r="B1208" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1208" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1208" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1208" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1208" t="n">
+        <v>700</v>
+      </c>
+      <c r="G1208" t="n">
+        <v>7979.543044930953</v>
+      </c>
+      <c r="H1208" t="n">
+        <v>7955.829434580442</v>
+      </c>
+      <c r="J1208" t="n">
+        <v>75788713258</v>
+      </c>
+    </row>
+    <row r="1209">
+      <c r="A1209" t="inlineStr">
+        <is>
+          <t>1000.30.1</t>
+        </is>
+      </c>
+      <c r="B1209" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1209" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1209" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1209" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1209" t="n">
+        <v>800</v>
+      </c>
+      <c r="G1209" t="n">
+        <v>7979.543044930953</v>
+      </c>
+      <c r="H1209" t="n">
+        <v>7922.295579699436</v>
+      </c>
+      <c r="J1209" t="n">
+        <v>75901553919</v>
+      </c>
+    </row>
+    <row r="1210">
+      <c r="A1210" t="inlineStr">
+        <is>
+          <t>1000.30.1</t>
+        </is>
+      </c>
+      <c r="B1210" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1210" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1210" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1210" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1210" t="n">
+        <v>900</v>
+      </c>
+      <c r="G1210" t="n">
+        <v>7979.543044930953</v>
+      </c>
+      <c r="H1210" t="n">
+        <v>7929.080911495736</v>
+      </c>
+      <c r="J1210" t="n">
+        <v>75863869312</v>
+      </c>
+    </row>
+    <row r="1211">
+      <c r="A1211" t="inlineStr">
+        <is>
+          <t>1000.30.1</t>
+        </is>
+      </c>
+      <c r="B1211" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1211" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1211" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1211" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1211" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G1211" t="n">
+        <v>7979.543044930953</v>
+      </c>
+      <c r="H1211" t="n">
+        <v>7925.45930514813</v>
+      </c>
+      <c r="J1211" t="n">
+        <v>75960176548</v>
+      </c>
+    </row>
+    <row r="1212">
+      <c r="A1212" t="inlineStr">
+        <is>
+          <t>1000.30.2</t>
+        </is>
+      </c>
+      <c r="B1212" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1212" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1212" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1212" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1212" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1212" t="n">
+        <v>7973.009423005142</v>
+      </c>
+      <c r="H1212" t="n">
+        <v>7955.478963396214</v>
+      </c>
+      <c r="I1212" t="n">
+        <v>7944.300020434308</v>
+      </c>
+      <c r="J1212" t="n">
+        <v>75463252430</v>
+      </c>
+      <c r="K1212" t="n">
+        <v>79665719147</v>
+      </c>
+    </row>
+    <row r="1213">
+      <c r="A1213" t="inlineStr">
+        <is>
+          <t>1000.30.2</t>
+        </is>
+      </c>
+      <c r="B1213" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1213" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1213" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1213" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1213" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1213" t="n">
+        <v>7973.009423005142</v>
+      </c>
+      <c r="H1213" t="n">
+        <v>7985.667796737807</v>
+      </c>
+      <c r="I1213" t="n">
+        <v>7950.033926181859</v>
+      </c>
+      <c r="J1213" t="n">
+        <v>75499709671</v>
+      </c>
+      <c r="K1213" t="n">
+        <v>79559486593</v>
+      </c>
+    </row>
+    <row r="1214">
+      <c r="A1214" t="inlineStr">
+        <is>
+          <t>1000.30.2</t>
+        </is>
+      </c>
+      <c r="B1214" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1214" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1214" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1214" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1214" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1214" t="n">
+        <v>7973.009423005142</v>
+      </c>
+      <c r="H1214" t="n">
+        <v>7971.863557246797</v>
+      </c>
+      <c r="I1214" t="n">
+        <v>7945.713457379617</v>
+      </c>
+      <c r="J1214" t="n">
+        <v>75291910014</v>
+      </c>
+      <c r="K1214" t="n">
+        <v>79646776106</v>
+      </c>
+    </row>
+    <row r="1215">
+      <c r="A1215" t="inlineStr">
+        <is>
+          <t>1000.30.2</t>
+        </is>
+      </c>
+      <c r="B1215" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1215" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1215" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1215" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1215" t="n">
+        <v>400</v>
+      </c>
+      <c r="G1215" t="n">
+        <v>7973.009423005142</v>
+      </c>
+      <c r="H1215" t="n">
+        <v>7969.203121317212</v>
+      </c>
+      <c r="I1215" t="n">
+        <v>7959.459092132034</v>
+      </c>
+      <c r="J1215" t="n">
+        <v>75090134651</v>
+      </c>
+      <c r="K1215" t="n">
+        <v>79191579668</v>
+      </c>
+    </row>
+    <row r="1216">
+      <c r="A1216" t="inlineStr">
+        <is>
+          <t>1000.30.2</t>
+        </is>
+      </c>
+      <c r="B1216" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1216" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1216" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1216" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1216" t="n">
+        <v>500</v>
+      </c>
+      <c r="G1216" t="n">
+        <v>7973.009423005142</v>
+      </c>
+      <c r="H1216" t="n">
+        <v>7979.309609375296</v>
+      </c>
+      <c r="I1216" t="n">
+        <v>7970.03120460759</v>
+      </c>
+      <c r="J1216" t="n">
+        <v>75328307082</v>
+      </c>
+      <c r="K1216" t="n">
+        <v>80012508520</v>
+      </c>
+    </row>
+    <row r="1217">
+      <c r="A1217" t="inlineStr">
+        <is>
+          <t>1000.30.2</t>
+        </is>
+      </c>
+      <c r="B1217" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1217" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1217" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1217" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1217" t="n">
+        <v>600</v>
+      </c>
+      <c r="G1217" t="n">
+        <v>7973.009423005142</v>
+      </c>
+      <c r="H1217" t="n">
+        <v>7971.19944637468</v>
+      </c>
+      <c r="J1217" t="n">
+        <v>75446297308</v>
+      </c>
+    </row>
+    <row r="1218">
+      <c r="A1218" t="inlineStr">
+        <is>
+          <t>1000.30.2</t>
+        </is>
+      </c>
+      <c r="B1218" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1218" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1218" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1218" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1218" t="n">
+        <v>700</v>
+      </c>
+      <c r="G1218" t="n">
+        <v>7973.009423005142</v>
+      </c>
+      <c r="H1218" t="n">
+        <v>7946.640807827146</v>
+      </c>
+      <c r="J1218" t="n">
+        <v>75276243496</v>
+      </c>
+    </row>
+    <row r="1219">
+      <c r="A1219" t="inlineStr">
+        <is>
+          <t>1000.30.2</t>
+        </is>
+      </c>
+      <c r="B1219" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1219" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1219" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1219" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1219" t="n">
+        <v>800</v>
+      </c>
+      <c r="G1219" t="n">
+        <v>7973.009423005142</v>
+      </c>
+      <c r="H1219" t="n">
+        <v>7987.275227344298</v>
+      </c>
+      <c r="J1219" t="n">
+        <v>75178609291</v>
+      </c>
+    </row>
+    <row r="1220">
+      <c r="A1220" t="inlineStr">
+        <is>
+          <t>1000.30.2</t>
+        </is>
+      </c>
+      <c r="B1220" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1220" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1220" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1220" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1220" t="n">
+        <v>900</v>
+      </c>
+      <c r="G1220" t="n">
+        <v>7973.009423005142</v>
+      </c>
+      <c r="H1220" t="n">
+        <v>7948.726835636515</v>
+      </c>
+      <c r="J1220" t="n">
+        <v>75465058292</v>
+      </c>
+    </row>
+    <row r="1221">
+      <c r="A1221" t="inlineStr">
+        <is>
+          <t>1000.30.2</t>
+        </is>
+      </c>
+      <c r="B1221" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1221" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1221" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1221" t="n">
+        <v>10</v>
+      </c>
+      <c r="F1221" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G1221" t="n">
+        <v>7973.009423005142</v>
+      </c>
+      <c r="H1221" t="n">
+        <v>7973.815100914153</v>
+      </c>
+      <c r="J1221" t="n">
+        <v>75293852541</v>
+      </c>
+    </row>
+    <row r="1222">
+      <c r="A1222" t="inlineStr">
+        <is>
+          <t>1000.30.3</t>
+        </is>
+      </c>
+      <c r="B1222" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1222" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1222" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1222" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1222" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1222" t="n">
+        <v>7977.814850915422</v>
+      </c>
+      <c r="H1222" t="n">
+        <v>7912.800374705674</v>
+      </c>
+      <c r="I1222" t="n">
+        <v>7920.722535902631</v>
+      </c>
+      <c r="J1222" t="n">
+        <v>75526679782</v>
+      </c>
+      <c r="K1222" t="n">
+        <v>79864223403</v>
+      </c>
+    </row>
+    <row r="1223">
+      <c r="A1223" t="inlineStr">
+        <is>
+          <t>1000.30.3</t>
+        </is>
+      </c>
+      <c r="B1223" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1223" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1223" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1223" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1223" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1223" t="n">
+        <v>7977.814850915422</v>
+      </c>
+      <c r="H1223" t="n">
+        <v>7920.286934325561</v>
+      </c>
+      <c r="I1223" t="n">
+        <v>7876.350396623391</v>
+      </c>
+      <c r="J1223" t="n">
+        <v>75239934410</v>
+      </c>
+      <c r="K1223" t="n">
+        <v>79854507057</v>
+      </c>
+    </row>
+    <row r="1224">
+      <c r="A1224" t="inlineStr">
+        <is>
+          <t>1000.30.3</t>
+        </is>
+      </c>
+      <c r="B1224" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1224" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1224" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1224" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1224" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1224" t="n">
+        <v>7977.814850915422</v>
+      </c>
+      <c r="H1224" t="n">
+        <v>7913.559085252405</v>
+      </c>
+      <c r="I1224" t="n">
+        <v>7860.33109598247</v>
+      </c>
+      <c r="J1224" t="n">
+        <v>75154106633</v>
+      </c>
+      <c r="K1224" t="n">
+        <v>79559590331</v>
+      </c>
+    </row>
+    <row r="1225">
+      <c r="A1225" t="inlineStr">
+        <is>
+          <t>1000.30.3</t>
+        </is>
+      </c>
+      <c r="B1225" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1225" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1225" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1225" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1225" t="n">
+        <v>400</v>
+      </c>
+      <c r="G1225" t="n">
+        <v>7977.814850915422</v>
+      </c>
+      <c r="H1225" t="n">
+        <v>7913.650487887249</v>
+      </c>
+      <c r="I1225" t="n">
+        <v>7920.365306495831</v>
+      </c>
+      <c r="J1225" t="n">
+        <v>75437065308</v>
+      </c>
+      <c r="K1225" t="n">
+        <v>79839038862</v>
+      </c>
+    </row>
+    <row r="1226">
+      <c r="A1226" t="inlineStr">
+        <is>
+          <t>1000.30.3</t>
+        </is>
+      </c>
+      <c r="B1226" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1226" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1226" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1226" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1226" t="n">
+        <v>500</v>
+      </c>
+      <c r="G1226" t="n">
+        <v>7977.814850915422</v>
+      </c>
+      <c r="H1226" t="n">
+        <v>7919.761908166192</v>
+      </c>
+      <c r="I1226" t="n">
+        <v>7864.197629346444</v>
+      </c>
+      <c r="J1226" t="n">
+        <v>75429078752</v>
+      </c>
+      <c r="K1226" t="n">
+        <v>79809132821</v>
+      </c>
+    </row>
+    <row r="1227">
+      <c r="A1227" t="inlineStr">
+        <is>
+          <t>1000.30.3</t>
+        </is>
+      </c>
+      <c r="B1227" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1227" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1227" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1227" t="n">
+        <v>6</v>
+      </c>
+      <c r="F1227" t="n">
+        <v>600</v>
+      </c>
+      <c r="G1227" t="n">
+        <v>7977.814850915422</v>
+      </c>
+      <c r="H1227" t="n">
+        <v>7880.649034908736</v>
+      </c>
+      <c r="J1227" t="n">
+        <v>67519046491</v>
+      </c>
+    </row>
+    <row r="1228">
+      <c r="A1228" t="inlineStr">
+        <is>
+          <t>1000.30.3</t>
+        </is>
+      </c>
+      <c r="B1228" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1228" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1228" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1228" t="n">
+        <v>7</v>
+      </c>
+      <c r="F1228" t="n">
+        <v>700</v>
+      </c>
+      <c r="G1228" t="n">
+        <v>7977.814850915422</v>
+      </c>
+      <c r="H1228" t="n">
+        <v>7898.118755099087</v>
+      </c>
+      <c r="J1228" t="n">
+        <v>73153473252</v>
+      </c>
+    </row>
+    <row r="1229">
+      <c r="A1229" t="inlineStr">
+        <is>
+          <t>1000.30.3</t>
+        </is>
+      </c>
+      <c r="B1229" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1229" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1229" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1229" t="n">
+        <v>8</v>
+      </c>
+      <c r="F1229" t="n">
+        <v>800</v>
+      </c>
+      <c r="G1229" t="n">
+        <v>7977.814850915422</v>
+      </c>
+      <c r="H1229" t="n">
+        <v>7865.5925004317</v>
+      </c>
+      <c r="J1229" t="n">
+        <v>75330589143</v>
+      </c>
+    </row>
+    <row r="1230">
+      <c r="A1230" t="inlineStr">
+        <is>
+          <t>1000.30.3</t>
+        </is>
+      </c>
+      <c r="B1230" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1230" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1230" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1230" t="n">
+        <v>9</v>
+      </c>
+      <c r="F1230" t="n">
+        <v>900</v>
+      </c>
+      <c r="G1230" t="n">
+        <v>7977.814850915422</v>
+      </c>
+      <c r="H1230" t="n">
+        <v>7870.972885162075</v>
+      </c>
+      <c r="J1230" t="n">
+        <v>75268039891</v>
+      </c>
+    </row>
+    <row r="1231">
+      <c r="A1231" t="inlineStr">
+        <is>
+          <t>1000.30.4</t>
+        </is>
+      </c>
+      <c r="B1231" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1231" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1231" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1231" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1231" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1231" t="n">
+        <v>7964.046250435393</v>
+      </c>
+      <c r="H1231" t="n">
+        <v>7954.622756722229</v>
+      </c>
+      <c r="I1231" t="n">
+        <v>7937.350316798198</v>
+      </c>
+      <c r="J1231" t="n">
+        <v>76298686901</v>
+      </c>
+      <c r="K1231" t="n">
+        <v>80345994552</v>
+      </c>
+    </row>
+    <row r="1232">
+      <c r="A1232" t="inlineStr">
+        <is>
+          <t>1000.30.4</t>
+        </is>
+      </c>
+      <c r="B1232" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1232" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1232" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1232" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1232" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1232" t="n">
+        <v>7964.046250435393</v>
+      </c>
+      <c r="H1232" t="n">
+        <v>7944.878378597256</v>
+      </c>
+      <c r="I1232" t="n">
+        <v>7945.437917149456</v>
+      </c>
+      <c r="J1232" t="n">
+        <v>76143958723</v>
+      </c>
+      <c r="K1232" t="n">
+        <v>80072300346</v>
+      </c>
+    </row>
+    <row r="1233">
+      <c r="A1233" t="inlineStr">
+        <is>
+          <t>1000.30.4</t>
+        </is>
+      </c>
+      <c r="B1233" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1233" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1233" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1233" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1233" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1233" t="n">
+        <v>7964.046250435393</v>
+      </c>
+      <c r="H1233" t="n">
+        <v>7908.149940826446</v>
+      </c>
+      <c r="I1233" t="n">
+        <v>7924.585067946708</v>
+      </c>
+      <c r="J1233" t="n">
+        <v>76310818841</v>
+      </c>
+      <c r="K1233" t="n">
+        <v>80329220533</v>
+      </c>
+    </row>
+    <row r="1234">
+      <c r="A1234" t="inlineStr">
+        <is>
+          <t>1000.30.4</t>
+        </is>
+      </c>
+      <c r="B1234" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1234" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1234" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1234" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1234" t="n">
+        <v>400</v>
+      </c>
+      <c r="G1234" t="n">
+        <v>7964.046250435393</v>
+      </c>
+      <c r="I1234" t="n">
+        <v>7929.577010942594</v>
+      </c>
+      <c r="K1234" t="n">
+        <v>79863930995</v>
+      </c>
+    </row>
+    <row r="1235">
+      <c r="A1235" t="inlineStr">
+        <is>
+          <t>1000.30.4</t>
+        </is>
+      </c>
+      <c r="B1235" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1235" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1235" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1235" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1235" t="n">
+        <v>500</v>
+      </c>
+      <c r="G1235" t="n">
+        <v>7964.046250435393</v>
+      </c>
+      <c r="I1235" t="n">
+        <v>7907.056895020358</v>
+      </c>
+      <c r="K1235" t="n">
+        <v>80221553843</v>
+      </c>
+    </row>
+    <row r="1236">
+      <c r="A1236" t="inlineStr">
+        <is>
+          <t>1000.40.1</t>
+        </is>
+      </c>
+      <c r="B1236" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1236" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1236" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1236" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1236" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1236" t="n">
+        <v>14005.02994874948</v>
+      </c>
+      <c r="H1236" t="n">
+        <v>13804.65911026816</v>
+      </c>
+      <c r="I1236" t="n">
+        <v>13727.06070999957</v>
+      </c>
+      <c r="J1236" t="n">
+        <v>85252367167</v>
+      </c>
+      <c r="K1236" t="n">
+        <v>87948448001</v>
+      </c>
+    </row>
+    <row r="1237">
+      <c r="A1237" t="inlineStr">
+        <is>
+          <t>1000.40.1</t>
+        </is>
+      </c>
+      <c r="B1237" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1237" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1237" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1237" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1237" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1237" t="n">
+        <v>14005.02994874948</v>
+      </c>
+      <c r="H1237" t="n">
+        <v>13703.5761313689</v>
+      </c>
+      <c r="I1237" t="n">
+        <v>13678.77539809002</v>
+      </c>
+      <c r="J1237" t="n">
+        <v>85000059396</v>
+      </c>
+      <c r="K1237" t="n">
+        <v>88387691033</v>
+      </c>
+    </row>
+    <row r="1238">
+      <c r="A1238" t="inlineStr">
+        <is>
+          <t>1000.40.1</t>
+        </is>
+      </c>
+      <c r="B1238" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1238" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1238" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1238" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1238" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1238" t="n">
+        <v>14005.02994874948</v>
+      </c>
+      <c r="H1238" t="n">
+        <v>13829.70485039924</v>
+      </c>
+      <c r="I1238" t="n">
+        <v>13707.46434839891</v>
+      </c>
+      <c r="J1238" t="n">
+        <v>84913861591</v>
+      </c>
+      <c r="K1238" t="n">
+        <v>88130654686</v>
+      </c>
+    </row>
+    <row r="1239">
+      <c r="A1239" t="inlineStr">
+        <is>
+          <t>1000.40.1</t>
+        </is>
+      </c>
+      <c r="B1239" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1239" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1239" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1239" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1239" t="n">
+        <v>400</v>
+      </c>
+      <c r="G1239" t="n">
+        <v>14005.02994874948</v>
+      </c>
+      <c r="I1239" t="n">
+        <v>13740.21554885748</v>
+      </c>
+      <c r="K1239" t="n">
+        <v>88297144687</v>
+      </c>
+    </row>
+    <row r="1240">
+      <c r="A1240" t="inlineStr">
+        <is>
+          <t>1000.40.1</t>
+        </is>
+      </c>
+      <c r="B1240" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1240" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1240" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1240" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1240" t="n">
+        <v>500</v>
+      </c>
+      <c r="G1240" t="n">
+        <v>14005.02994874948</v>
+      </c>
+      <c r="I1240" t="n">
+        <v>13666.85921821061</v>
+      </c>
+      <c r="K1240" t="n">
+        <v>88392609632</v>
+      </c>
+    </row>
+    <row r="1241">
+      <c r="A1241" t="inlineStr">
+        <is>
+          <t>1000.40.2</t>
+        </is>
+      </c>
+      <c r="B1241" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1241" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1241" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1241" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1241" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1241" t="n">
+        <v>14118.04105210099</v>
+      </c>
+      <c r="H1241" t="n">
+        <v>13953.57733794516</v>
+      </c>
+      <c r="I1241" t="n">
+        <v>13931.39017551439</v>
+      </c>
+      <c r="J1241" t="n">
+        <v>84476830074</v>
+      </c>
+      <c r="K1241" t="n">
+        <v>88463191445</v>
+      </c>
+    </row>
+    <row r="1242">
+      <c r="A1242" t="inlineStr">
+        <is>
+          <t>1000.40.2</t>
+        </is>
+      </c>
+      <c r="B1242" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1242" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1242" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1242" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1242" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1242" t="n">
+        <v>14118.04105210099</v>
+      </c>
+      <c r="H1242" t="n">
+        <v>13879.86269944144</v>
+      </c>
+      <c r="I1242" t="n">
+        <v>13850.72930858321</v>
+      </c>
+      <c r="J1242" t="n">
+        <v>84567750703</v>
+      </c>
+      <c r="K1242" t="n">
+        <v>88374159109</v>
+      </c>
+    </row>
+    <row r="1243">
+      <c r="A1243" t="inlineStr">
+        <is>
+          <t>1000.40.2</t>
+        </is>
+      </c>
+      <c r="B1243" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1243" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1243" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1243" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1243" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1243" t="n">
+        <v>14118.04105210099</v>
+      </c>
+      <c r="H1243" t="n">
+        <v>13960.02681644472</v>
+      </c>
+      <c r="I1243" t="n">
+        <v>13917.82365179558</v>
+      </c>
+      <c r="J1243" t="n">
+        <v>84895471386</v>
+      </c>
+      <c r="K1243" t="n">
+        <v>88267450156</v>
+      </c>
+    </row>
+    <row r="1244">
+      <c r="A1244" t="inlineStr">
+        <is>
+          <t>1000.40.2</t>
+        </is>
+      </c>
+      <c r="B1244" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1244" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1244" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1244" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1244" t="n">
+        <v>400</v>
+      </c>
+      <c r="G1244" t="n">
+        <v>14118.04105210099</v>
+      </c>
+      <c r="I1244" t="n">
+        <v>13860.35154425662</v>
+      </c>
+      <c r="K1244" t="n">
+        <v>88312094525</v>
+      </c>
+    </row>
+    <row r="1245">
+      <c r="A1245" t="inlineStr">
+        <is>
+          <t>1000.40.2</t>
+        </is>
+      </c>
+      <c r="B1245" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1245" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1245" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1245" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1245" t="n">
+        <v>500</v>
+      </c>
+      <c r="G1245" t="n">
+        <v>14118.04105210099</v>
+      </c>
+      <c r="I1245" t="n">
+        <v>13816.65492916855</v>
+      </c>
+      <c r="K1245" t="n">
+        <v>88256861778</v>
+      </c>
+    </row>
+    <row r="1246">
+      <c r="A1246" t="inlineStr">
+        <is>
+          <t>1000.40.3</t>
+        </is>
+      </c>
+      <c r="B1246" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1246" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1246" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1246" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1246" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1246" t="n">
+        <v>14052.70747046845</v>
+      </c>
+      <c r="H1246" t="n">
+        <v>13928.43424030587</v>
+      </c>
+      <c r="I1246" t="n">
+        <v>13866.49181471369</v>
+      </c>
+      <c r="J1246" t="n">
+        <v>84955360440</v>
+      </c>
+      <c r="K1246" t="n">
+        <v>88491758334</v>
+      </c>
+    </row>
+    <row r="1247">
+      <c r="A1247" t="inlineStr">
+        <is>
+          <t>1000.40.3</t>
+        </is>
+      </c>
+      <c r="B1247" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1247" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1247" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1247" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1247" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1247" t="n">
+        <v>14052.70747046845</v>
+      </c>
+      <c r="H1247" t="n">
+        <v>14025.13225262927</v>
+      </c>
+      <c r="I1247" t="n">
+        <v>13992.15523571734</v>
+      </c>
+      <c r="J1247" t="n">
+        <v>84845024911</v>
+      </c>
+      <c r="K1247" t="n">
+        <v>88258794676</v>
+      </c>
+    </row>
+    <row r="1248">
+      <c r="A1248" t="inlineStr">
+        <is>
+          <t>1000.40.3</t>
+        </is>
+      </c>
+      <c r="B1248" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1248" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1248" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1248" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1248" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1248" t="n">
+        <v>14052.70747046845</v>
+      </c>
+      <c r="H1248" t="n">
+        <v>13988.34944155203</v>
+      </c>
+      <c r="I1248" t="n">
+        <v>13922.58586497711</v>
+      </c>
+      <c r="J1248" t="n">
+        <v>85041302241</v>
+      </c>
+      <c r="K1248" t="n">
+        <v>88291746606</v>
+      </c>
+    </row>
+    <row r="1249">
+      <c r="A1249" t="inlineStr">
+        <is>
+          <t>1000.40.3</t>
+        </is>
+      </c>
+      <c r="B1249" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1249" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1249" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1249" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1249" t="n">
+        <v>400</v>
+      </c>
+      <c r="G1249" t="n">
+        <v>14052.70747046845</v>
+      </c>
+      <c r="I1249" t="n">
+        <v>13985.74834269132</v>
+      </c>
+      <c r="K1249" t="n">
+        <v>88070207994</v>
+      </c>
+    </row>
+    <row r="1250">
+      <c r="A1250" t="inlineStr">
+        <is>
+          <t>1000.40.3</t>
+        </is>
+      </c>
+      <c r="B1250" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1250" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1250" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1250" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1250" t="n">
+        <v>500</v>
+      </c>
+      <c r="G1250" t="n">
+        <v>14052.70747046845</v>
+      </c>
+      <c r="I1250" t="n">
+        <v>13920.36568946934</v>
+      </c>
+      <c r="K1250" t="n">
+        <v>88382124558</v>
+      </c>
+    </row>
+    <row r="1251">
+      <c r="A1251" t="inlineStr">
+        <is>
+          <t>1000.40.4</t>
+        </is>
+      </c>
+      <c r="B1251" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1251" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1251" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1251" t="n">
+        <v>1</v>
+      </c>
+      <c r="F1251" t="n">
+        <v>100</v>
+      </c>
+      <c r="G1251" t="n">
         <v>14047.58679159633</v>
       </c>
-      <c r="I1201" t="n">
+      <c r="H1251" t="n">
+        <v>13855.13481452877</v>
+      </c>
+      <c r="I1251" t="n">
+        <v>13769.51168139956</v>
+      </c>
+      <c r="J1251" t="n">
+        <v>84108180671</v>
+      </c>
+      <c r="K1251" t="n">
+        <v>88169613935</v>
+      </c>
+    </row>
+    <row r="1252">
+      <c r="A1252" t="inlineStr">
+        <is>
+          <t>1000.40.4</t>
+        </is>
+      </c>
+      <c r="B1252" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1252" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1252" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1252" t="n">
+        <v>2</v>
+      </c>
+      <c r="F1252" t="n">
+        <v>200</v>
+      </c>
+      <c r="G1252" t="n">
+        <v>14047.58679159633</v>
+      </c>
+      <c r="H1252" t="n">
+        <v>13808.05311567009</v>
+      </c>
+      <c r="I1252" t="n">
+        <v>13792.0484138216</v>
+      </c>
+      <c r="J1252" t="n">
+        <v>83932164076</v>
+      </c>
+      <c r="K1252" t="n">
+        <v>87849710144</v>
+      </c>
+    </row>
+    <row r="1253">
+      <c r="A1253" t="inlineStr">
+        <is>
+          <t>1000.40.4</t>
+        </is>
+      </c>
+      <c r="B1253" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1253" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1253" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1253" t="n">
+        <v>3</v>
+      </c>
+      <c r="F1253" t="n">
+        <v>300</v>
+      </c>
+      <c r="G1253" t="n">
+        <v>14047.58679159633</v>
+      </c>
+      <c r="H1253" t="n">
+        <v>13788.06577326823</v>
+      </c>
+      <c r="I1253" t="n">
+        <v>13833.52844773018</v>
+      </c>
+      <c r="J1253" t="n">
+        <v>84099856887</v>
+      </c>
+      <c r="K1253" t="n">
+        <v>88168171393</v>
+      </c>
+    </row>
+    <row r="1254">
+      <c r="A1254" t="inlineStr">
+        <is>
+          <t>1000.40.4</t>
+        </is>
+      </c>
+      <c r="B1254" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1254" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1254" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1254" t="n">
+        <v>4</v>
+      </c>
+      <c r="F1254" t="n">
+        <v>400</v>
+      </c>
+      <c r="G1254" t="n">
+        <v>14047.58679159633</v>
+      </c>
+      <c r="I1254" t="n">
+        <v>13774.94086040058</v>
+      </c>
+      <c r="K1254" t="n">
+        <v>87919633198</v>
+      </c>
+    </row>
+    <row r="1255">
+      <c r="A1255" t="inlineStr">
+        <is>
+          <t>1000.40.4</t>
+        </is>
+      </c>
+      <c r="B1255" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C1255" t="inlineStr">
+        <is>
+          <t>held-out</t>
+        </is>
+      </c>
+      <c r="D1255" t="n">
+        <v>4500</v>
+      </c>
+      <c r="E1255" t="n">
+        <v>5</v>
+      </c>
+      <c r="F1255" t="n">
+        <v>500</v>
+      </c>
+      <c r="G1255" t="n">
+        <v>14047.58679159633</v>
+      </c>
+      <c r="I1255" t="n">
         <v>13832.13975302853</v>
       </c>
-      <c r="K1201" t="n">
+      <c r="K1255" t="n">
         <v>87930082279</v>
       </c>
     </row>

</xml_diff>